<commit_message>
Revised the formula for construction
</commit_message>
<xml_diff>
--- a/InputData/io-model/BObIC/BAU Output by ISIC Code.xlsx
+++ b/InputData/io-model/BObIC/BAU Output by ISIC Code.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saido\OneDrive\Documents\eps-brazil-cpl\InputData\io-model\BObIC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saido\Documents\eps-brazil-cpl\InputData\io-model\BObIC\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -9059,8 +9059,8 @@
         <v>57763254487.389854</v>
       </c>
       <c r="AC2" s="81">
-        <f>'OECD TTL'!X30*10^6*About!A30</f>
-        <v>132321902.64833325</v>
+        <f>'OECD TTL'!X49*10^6*About!$A$30</f>
+        <v>1309373273311.197</v>
       </c>
       <c r="AD2">
         <f>'OECD TTL'!Y49*10^6*About!$A$30</f>

</xml_diff>